<commit_message>
modif intermediaire interface graphique
</commit_message>
<xml_diff>
--- a/PM_Garches.xlsx
+++ b/PM_Garches.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -871,12 +871,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Clinique du Château</t>
+          <t>Chapelle</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>hôpital</t>
+          <t>lieu de culte</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -885,26 +885,26 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>48.8437234</v>
+        <v>48.8390784</v>
       </c>
       <c r="E17" t="n">
-        <v>2.1970011</v>
+        <v>2.16866</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>48.8437234, 2.1970011</t>
+          <t>48.8390784, 2.16866</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hôpital Raymond Poincaré</t>
+          <t>Église Saint-Louis</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>hôpital</t>
+          <t>lieu de culte</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -913,54 +913,54 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>48.8393703</v>
+        <v>48.8448446</v>
       </c>
       <c r="E18" t="n">
-        <v>2.1694837</v>
+        <v>2.1879912</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>48.8393703, 2.1694837</t>
+          <t>48.8448446, 2.1879912</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Protection Civile de Garches</t>
+          <t>Mairie - Garches</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>hôpital</t>
+          <t>mairie</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OpenStreetMap</t>
+          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>48.8516199</v>
+        <v>48.843436</v>
       </c>
       <c r="E19" t="n">
-        <v>2.1976296</v>
+        <v>2.187209</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>48.8516199, 2.1976296</t>
+          <t>48.843436, 2.187209</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Chapelle</t>
+          <t>Para &amp; Pharmacie de la gare</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>lieu de culte</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -969,26 +969,26 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>48.8390784</v>
+        <v>48.8392672</v>
       </c>
       <c r="E20" t="n">
-        <v>2.16866</v>
+        <v>2.1859957</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>48.8390784, 2.16866</t>
+          <t>48.8392672, 2.1859957</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Église Saint-Louis</t>
+          <t>Pharmacie Pasteur</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>lieu de culte</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -997,49 +997,49 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>48.8448446</v>
+        <v>48.8410092</v>
       </c>
       <c r="E21" t="n">
-        <v>2.1879912</v>
+        <v>2.1813105</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>48.8448446, 2.1879912</t>
+          <t>48.8410092, 2.1813105</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mairie - Garches</t>
+          <t>Pharmacie de L'Hôtel de Ville</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>mairie</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
+          <t>OpenStreetMap</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>48.843436</v>
+        <v>48.8438141</v>
       </c>
       <c r="E22" t="n">
-        <v>2.187209</v>
+        <v>2.186653</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>48.843436, 2.187209</t>
+          <t>48.8438141, 2.186653</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Para &amp; Pharmacie de la gare</t>
+          <t>Pharmacie de la Verboise</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1053,21 +1053,21 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>48.8392672</v>
+        <v>48.8473975</v>
       </c>
       <c r="E23" t="n">
-        <v>2.1859957</v>
+        <v>2.1957291</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>48.8392672, 2.1859957</t>
+          <t>48.8473975, 2.1957291</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pharmacie Pasteur</t>
+          <t>Pharmacie du Golf</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1081,21 +1081,21 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>48.8410092</v>
+        <v>48.8491703</v>
       </c>
       <c r="E24" t="n">
-        <v>2.1813105</v>
+        <v>2.2010502</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>48.8410092, 2.1813105</t>
+          <t>48.8491703, 2.2010502</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Pharmacie de L'Hôtel de Ville</t>
+          <t>Pharmacie du Marché Saint-Louis</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1109,26 +1109,26 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>48.8438141</v>
+        <v>48.844952</v>
       </c>
       <c r="E25" t="n">
-        <v>2.186653</v>
+        <v>2.1869709</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>48.8438141, 2.186653</t>
+          <t>48.844952, 2.1869709</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Pharmacie de la Verboise</t>
+          <t>Garches</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>pharmacie</t>
+          <t>poste</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1137,26 +1137,26 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>48.8473975</v>
+        <v>48.8439718</v>
       </c>
       <c r="E26" t="n">
-        <v>2.1957291</v>
+        <v>2.1851004</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>48.8473975, 2.1957291</t>
+          <t>48.8439718, 2.1851004</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pharmacie du Golf</t>
+          <t>G20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>pharmacie</t>
+          <t>supermarché</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1165,26 +1165,26 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>48.8491703</v>
+        <v>48.8389899</v>
       </c>
       <c r="E27" t="n">
-        <v>2.2010502</v>
+        <v>2.1871146</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>48.8491703, 2.2010502</t>
+          <t>48.8389899, 2.1871146</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pharmacie du Marché Saint-Louis</t>
+          <t>Monoprix</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>pharmacie</t>
+          <t>supermarché</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1193,26 +1193,26 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>48.844952</v>
+        <v>48.8389242</v>
       </c>
       <c r="E28" t="n">
-        <v>2.1869709</v>
+        <v>2.1865652</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>48.844952, 2.1869709</t>
+          <t>48.8389242, 2.1865652</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Garches</t>
+          <t>Super U</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>supermarché</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1221,96 +1221,12 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>48.8439718</v>
+        <v>48.8455949</v>
       </c>
       <c r="E29" t="n">
-        <v>2.1851004</v>
+        <v>2.1887469</v>
       </c>
       <c r="F29" t="inlineStr">
-        <is>
-          <t>48.8439718, 2.1851004</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>G20</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>supermarché</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>48.8389899</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2.1871146</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>48.8389899, 2.1871146</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Monoprix</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>supermarché</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>48.8389242</v>
-      </c>
-      <c r="E31" t="n">
-        <v>2.1865652</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>48.8389242, 2.1865652</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Super U</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>supermarché</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>48.8455949</v>
-      </c>
-      <c r="E32" t="n">
-        <v>2.1887469</v>
-      </c>
-      <c r="F32" t="inlineStr">
         <is>
           <t>48.8455949, 2.1887469</t>
         </is>

</xml_diff>